<commit_message>
Added Opportunity and Leads Module POM classes, Test Scripts, XML files.
</commit_message>
<xml_diff>
--- a/vTiger1/src/test/resources/TestData.xlsx
+++ b/vTiger1/src/test/resources/TestData.xlsx
@@ -5,16 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\eclipse-workspace\vTiger\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\git\repository5\vTiger1\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5BD80F5-C102-494C-96C5-F3B1B7F34FB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6BC70A02-588F-47BE-B1C6-393BE08EB823}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1284" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Organization" sheetId="1" r:id="rId1"/>
     <sheet name="Contacts" sheetId="2" r:id="rId2"/>
+    <sheet name="Opportunities" sheetId="3" r:id="rId3"/>
+    <sheet name="Leads" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="33">
   <si>
     <t>Organization Name</t>
   </si>
@@ -71,6 +73,60 @@
   </si>
   <si>
     <t>End Date</t>
+  </si>
+  <si>
+    <t>Opportunity Name</t>
+  </si>
+  <si>
+    <t>Peter Parker</t>
+  </si>
+  <si>
+    <t>Bruce Wayne</t>
+  </si>
+  <si>
+    <t>Clark Kent</t>
+  </si>
+  <si>
+    <t>Related To</t>
+  </si>
+  <si>
+    <t>Organizations</t>
+  </si>
+  <si>
+    <t>Contacts</t>
+  </si>
+  <si>
+    <t>Sales Stage</t>
+  </si>
+  <si>
+    <t>Needs Analysis</t>
+  </si>
+  <si>
+    <t>Qualification</t>
+  </si>
+  <si>
+    <t>Proposal/Price Quote</t>
+  </si>
+  <si>
+    <t>Lead name</t>
+  </si>
+  <si>
+    <t>Company Name</t>
+  </si>
+  <si>
+    <t>Mobile</t>
+  </si>
+  <si>
+    <t>Stark Industries</t>
+  </si>
+  <si>
+    <t>Electronics</t>
+  </si>
+  <si>
+    <t>Wayne Enterprises</t>
+  </si>
+  <si>
+    <t>Tony Stark</t>
   </si>
 </sst>
 </file>
@@ -391,7 +447,7 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
   </cols>
@@ -451,9 +507,8 @@
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
@@ -504,4 +559,133 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB2524BE-C24E-4267-A3C9-6C8C183D90E7}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2">
+        <v>30</v>
+      </c>
+      <c r="D2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3">
+        <v>45</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4">
+        <v>60</v>
+      </c>
+      <c r="D4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF9223FB-4715-4506-853A-D791280DB458}">
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>29</v>
+      </c>
+      <c r="C2">
+        <v>9874563210</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3">
+        <v>9632587410</v>
+      </c>
+      <c r="D3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>